<commit_message>
fix(mdx): bo sung day du cot Goals va cac file thuc thi cho Query 07 va Query 09 len github
</commit_message>
<xml_diff>
--- a/Bao_Cao_Double_Check_Query_10_11.xlsx
+++ b/Bao_Cao_Double_Check_Query_10_11.xlsx
@@ -10,6 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query 04 - Hieu Suat Do Tuoi" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query 10 - QoQ Top 10 CLB" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query 11 - Sân trên 60k Chỗ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query 07 - Pareto Ban Thang Anh" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query 09 - Intersect 9 CLB" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -99,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,6 +160,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -526,7 +534,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
@@ -549,7 +557,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1088,7 +1095,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -1484,7 +1491,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="101" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
@@ -2095,4 +2102,616 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="126" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BÁO CÁO PHÂN TÍCH PARETO 80/20 BÀN THẮNG THEO QUỐC TỊCH - CÁC GIẢI ĐẤU NƯỚC ANH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Nguồn dữ liệu: SSAS Cube [DW Football Transfermarkt] | Đối tượng: [DIM Player].[Country Of Citizenship], [DIM Competition]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Quốc Tịch (Country Of Citizenship)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Tổng Bàn Thắng (Goals)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Tỷ Lệ Đóng Góp (% England Goals)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>714</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>0.3193202146690519</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>194</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>0.08676207513416816</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>91</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>0.04069767441860465</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>89</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>0.03980322003577817</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>86</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>0.03846153846153846</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>79</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>0.0353309481216458</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>0.02415026833631485</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>53</v>
+      </c>
+      <c r="D12" s="23" t="n">
+        <v>0.02370304114490161</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>52</v>
+      </c>
+      <c r="D13" s="22" t="n">
+        <v>0.02325581395348837</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>51</v>
+      </c>
+      <c r="D14" s="23" t="n">
+        <v>0.02280858676207513</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>51</v>
+      </c>
+      <c r="D15" s="22" t="n">
+        <v>0.02280858676207513</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>48</v>
+      </c>
+      <c r="D16" s="23" t="n">
+        <v>0.02146690518783542</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Jamaica</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="D17" s="22" t="n">
+        <v>0.01967799642218247</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Korea, South</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>42</v>
+      </c>
+      <c r="D18" s="23" t="n">
+        <v>0.01878354203935599</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="D19" s="22" t="n">
+        <v>0.01744186046511628</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>37</v>
+      </c>
+      <c r="D20" s="23" t="n">
+        <v>0.0165474060822898</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="D21" s="22" t="n">
+        <v>0.0165474060822898</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D22" s="23" t="n">
+        <v>0.01565295169946333</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="117" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BÁO CÁO GIAO TẬP HỢP INTERSECT TOP 30 CLB XUẤT SẮC CẢ CUỐI TUẦN &amp; NGÀY THƯỜNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Nguồn dữ liệu: SSAS Cube [DW Football Transfermarkt] | Đối tượng: [DIM Club].[Club Name], [DIM Time].[Is Weekend]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Tên Câu Lạc Bộ (Club Name)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Cuối tuần - Bàn Thắng (Goals)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Cuối tuần - Thẻ Vàng</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Ngày thường - Bàn Thắng (Goals)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Ngày thường - Thẻ Vàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>94</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>49</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>151</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>115</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>62</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>110</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>137</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>76</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>47</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>134</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Arsenal FC</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>124</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>59</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>139</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Bayer 04 Leverkusen</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>65</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>74</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>126</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Celtic FC</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>43</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>111</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Inter Milan</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>49</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>114</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>103</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>